<commit_message>
Replace forecast table with primary-source data (ЦБ РФ, SberCIB, Эксперт РА, ВТБ, ДОМ.РФ)
Заменил ссылки на пересказы СМИ прямыми ссылками на первоисточники: официальные документы cbr.ru, sbercib.ru, raexpert.ru, прямую цитату ВТБ (ПМЭФ-2026) и офиц. пост ДОМ.РФ.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Прогнозы банков по ипотеке.xlsx
+++ b/Прогнозы банков по ипотеке.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прогнозы ипотеки" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прогнозы (первоисточники)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Прогнозы ипотеки'!$A$1:$F$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Прогнозы (первоисточники)'!$A$1:$H$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,15 +431,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -450,27 +452,37 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Тип источника</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Показатель</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Период прогноза</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Сценарий</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Прогнозное значение</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Сценарий / примечание</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Ссылка на источник</t>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Дата публикации</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Ссылка на первоисточник</t>
         </is>
       </c>
     </row>
@@ -482,27 +494,37 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>Первичный — офиц. документ</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>Ключевая ставка (среднегодовая)</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Базовый</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>14,5–14,6%</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Базовый сценарий</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>https://lenta.ru/news/2026/08/31/bank-rossii-predskazal-klyuchevuyu-stavku-na-blizhayshie-gody/</t>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>31.08.2026</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
         </is>
       </c>
     </row>
@@ -514,27 +536,37 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>Первичный — офиц. документ</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>Ключевая ставка (среднегодовая)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>2027</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Базовый</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>10,5–12,5%</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Базовый сценарий</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>https://lenta.ru/news/2026/08/31/bank-rossii-predskazal-klyuchevuyu-stavku-na-blizhayshie-gody/</t>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>31.08.2026</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
         </is>
       </c>
     </row>
@@ -546,27 +578,37 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
+          <t>Первичный — офиц. документ</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
           <t>Ключевая ставка (среднегодовая)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>2028</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>8–9%</t>
-        </is>
-      </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Базовый сценарий</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://lenta.ru/news/2026/08/31/bank-rossii-predskazal-klyuchevuyu-stavku-na-blizhayshie-gody/</t>
+          <t>8,0–9,0%</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>31.08.2026</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
         </is>
       </c>
     </row>
@@ -578,475 +620,625 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
+          <t>Первичный — офиц. документ</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
           <t>Ключевая ставка (среднегодовая)</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>2029</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Базовый</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>7,5–8,5%</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Базовый сценарий</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>https://lenta.ru/news/2026/08/31/bank-rossii-predskazal-klyuchevuyu-stavku-na-blizhayshie-gody/</t>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>31.08.2026</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>SberCIB</t>
+          <t>Банк России (ЦБ РФ)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка</t>
+          <t>Первичный — офиц. документ</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Сентябрь 2026</t>
+          <t>Ключевая ставка (среднегодовая)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>2027</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Базовый сценарий, помесячный прогноз</t>
+          <t>Дезинфляционный</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
+          <t>9,0–11,0%</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>31.08.2026</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>SberCIB</t>
+          <t>Банк России (ЦБ РФ)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка</t>
+          <t>Первичный — офиц. документ</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Октябрь 2026</t>
+          <t>Ключевая ставка (среднегодовая)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>13,75%</t>
+          <t>2027</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Базовый сценарий, помесячный прогноз</t>
+          <t>Проинфляционный</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
+          <t>13,0–15,0%</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>31.08.2026</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>SberCIB</t>
+          <t>Банк России (ЦБ РФ)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка</t>
+          <t>Первичный — офиц. документ</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Ноябрь 2026</t>
+          <t>Ключевая ставка (среднегодовая)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>13,75%</t>
+          <t>2027</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Базовый сценарий, помесячный прогноз</t>
+          <t>Рисковый</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
+          <t>19,0–21,0%</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>31.08.2026</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>SberCIB</t>
+          <t>Банк России (ЦБ РФ)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка</t>
+          <t>Первичный — офиц. документ (более ранняя оценка)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Декабрь 2026</t>
+          <t>Ключевая ставка (среднегодовая)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>13,5%</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Базовый сценарий, помесячный прогноз</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
+          <t>14,0–14,5%</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>07.05.2026</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/dkp/mp_dec/decision_key_rate/comment_07052026/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>SberCIB</t>
+          <t>Банк России (ЦБ РФ)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
+          <t>Первичный — офиц. документ (более ранняя оценка)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
           <t>Ключевая ставка (среднегодовая)</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>14,5%</t>
+          <t>2027</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Базовый сценарий</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
+          <t>8,0–10,0%</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>07.05.2026</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/dkp/mp_dec/decision_key_rate/comment_07052026/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>ВТБ</t>
+          <t>Банк России (ЦБ РФ)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Объём рыночной ипотеки (выдачи)</t>
+          <t>Первичный — офиц. документ (более ранняя оценка)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>Ключевая ставка (среднегодовая)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>~2,4 трлн руб.</t>
+          <t>2028</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Рост рынка +16% г/г</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>https://finance.mail.ru/article/vtb-prognoziruet-rost-rynochnoj-ipoteki-v-rossii-v-2026-godu-69225626/</t>
+          <t>7,5–8,5%</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>07.05.2026</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/dkp/mp_dec/decision_key_rate/comment_07052026/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ВТБ</t>
+          <t>Банк России (ЦБ РФ)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Рост ипотечного рынка</t>
+          <t>Первичный — офиц. документ (предыдущий цикл)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
+          <t>Ключевая ставка (среднегодовая)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>+16%</t>
-        </is>
-      </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>г/г</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>https://brief24.ru/news/2026/9/2/298933</t>
+          <t>13,0–15,0%</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>н/д (ОНЕДКП 2026-2028)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2026_2028/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>ВТБ</t>
+          <t>Банк России (ЦБ РФ)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Ставки по жилищным кредитам</t>
+          <t>Первичный — офиц. документ (предыдущий цикл)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Июнь 2026</t>
+          <t>Ключевая ставка (среднегодовая)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Без изменений</t>
+          <t>2027</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Факт на дату публикации, а не прогноз</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>https://finance.mail.ru/article/rossijskie-banki-poka-ne-toropyatsya-massovo-menyat-usloviya-po-ipoteke-69214403/</t>
+          <t>7,5–8,5%</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>н/д (ОНЕДКП 2026-2028)</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2026_2028/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Сбербанк</t>
+          <t>SberCIB (аналитика Сбербанка)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Ставки по жилищным кредитам</t>
+          <t>Первичный — сайт SberCIB</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Июнь 2026</t>
+          <t>Ключевая ставка</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Без изменений</t>
+          <t>Сентябрь 2026</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Факт на дату публикации, а не прогноз</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>https://finance.mail.ru/article/rossijskie-banki-poka-ne-toropyatsya-massovo-menyat-usloviya-po-ipoteke-69214403/</t>
+          <t>14%</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>н/д (публикация действует на 2026 год)</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Дом.РФ</t>
+          <t>SberCIB (аналитика Сбербанка)</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Объём выдач ипотеки</t>
+          <t>Первичный — сайт SberCIB</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>Ключевая ставка</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>~1,1 млн кредитов / 4,6 трлн руб.</t>
+          <t>Октябрь 2026</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Базовый прогноз</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>https://xn--h1alcedd.xn--d1aqf.xn--p1ai/instructions/rynochnaya-ipoteka/</t>
+          <t>13,75%</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>н/д</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Дом.РФ</t>
+          <t>SberCIB (аналитика Сбербанка)</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Ставка на первичном рынке</t>
+          <t>Первичный — сайт SberCIB</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Конец 2026</t>
+          <t>Ключевая ставка</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>до ~15%</t>
+          <t>Ноябрь 2026</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Наиболее реалистичный сценарий</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>https://xn--h1alcedd.xn--d1aqf.xn--p1ai/instructions/rynochnaya-ipoteka/</t>
+          <t>13,75%</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>н/д</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Дом.РФ</t>
+          <t>SberCIB (аналитика Сбербанка)</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Ставка по рыночной ипотеке</t>
+          <t>Первичный — сайт SberCIB</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>Ключевая ставка</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>до 10% и ниже</t>
+          <t>Декабрь 2026</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Ожидается кратный рост спроса, цены +10–15%</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>https://realty.ria.ru/20251202/ipoteka-2058963757.html</t>
+          <t>13,5%</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>н/д</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Совкомбанк</t>
+          <t>SberCIB (аналитика Сбербанка)</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка ЦБ</t>
+          <t>Первичный — сайт SberCIB</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Конец 2026</t>
+          <t>Ключевая ставка (среднегодовая)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>до 12%</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Более активный рост выдач ипотеки во 2-м полугодии</t>
+          <t>Базовый</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>https://realty.rbc.ru/news/69b41c839a7947ae12db0186</t>
+          <t>14,5%</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>н/д</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Минфин РФ</t>
+          <t>Эксперт РА</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Ставки по ипотеке</t>
+          <t>Первичный — исследование агентства</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
+          <t>Объём выдач ипотеки</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>снижение на 4–5 п.п. (примерно до 16–17%)</t>
-        </is>
-      </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Ведомственная оценка</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>https://realty.ria.ru/20251202/ipoteka-2058963757.html</t>
+          <t>Рост на 15–20% г/г, свыше 5 трлн руб.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>н/д</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>https://raexpert.ru/researches/banks/ipoteka_2026/</t>
         </is>
       </c>
     </row>
@@ -1058,19 +1250,19 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Ставки по ипотеке</t>
+          <t>Первичный — исследование агентства</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
+          <t>Доля льготной ипотеки в выдачах</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
           <t>1-е полугодие 2026</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>17–21%</t>
-        </is>
-      </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -1078,7 +1270,17 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>https://www.novostroy-m.ru/statyi/ipoteka_2026</t>
+          <t>Выше 50%</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>н/д</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>https://raexpert.ru/researches/banks/ipoteka_2026/</t>
         </is>
       </c>
     </row>
@@ -1090,96 +1292,252 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Ставки по ипотеке</t>
+          <t>Первичный — исследование агентства</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
+          <t>Доля льготной ипотеки в выдачах</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
           <t>2-е полугодие 2026</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>~15–16%</t>
-        </is>
-      </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>При условии ускорения смягчения ДКП со 2-го полугодия</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>https://www.novostroy-m.ru/statyi/ipoteka_2026</t>
+          <t>Паритет с рыночной (~50%)</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>н/д</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>https://raexpert.ru/researches/banks/ipoteka_2026/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Frank RG / отраслевые аналитики</t>
+          <t>Эксперт РА</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Объём выдач ипотеки (рынок в целом)</t>
+          <t>Первичный — исследование агентства (др. отчёт)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
+          <t>Объём выдач ипотеки</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>1–1,2 млн кредитов / 4,5–5 трлн руб.</t>
-        </is>
-      </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Агрегированная оценка рынка</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>https://frankrg.com/news/ipoteka-2025-2026-stress-test-vysokimi-stavkami-i-prognozy-na-vosstanovlenie</t>
+          <t>До 6,2 трлн руб. (1,2 млн кредитов), +59% г/г</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>н/д</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>https://raexpert.ru/researches/banks/bank_forecast_2026/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Рынок (справочно, факт)</t>
+          <t>Эксперт РА</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Средневзвешенная ставка по ипотеке</t>
+          <t>Первичный — исследование агентства (др. отчёт, для сравнения)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Сентябрь 2026</t>
+          <t>Объём выдач ипотеки</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>~18,5% (диапазон 15,9–19,45%)</t>
+          <t>2025 (факт/оценка)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Факт на дату публикации, а не прогноз</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>https://xn--h1alcedd.xn--d1aqf.xn--p1ai/news/obzor-stavok-po-ipoteke-v-bankakh-na-2-sentyabrya-2026-goda/</t>
+          <t>3,9 трлн руб., −20% г/г</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>н/д</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>https://raexpert.ru/researches/banks/bank_forecast_2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>ВТБ</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — прямая цитата официального лица (ст. вице-президент А. Охорзин), ПМЭФ-2026; зафиксировано информагентством ПРАЙМ, т.к. отдельного пресс-релиза на vtb.ru не найдено</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Объём выдач ипотеки</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>&gt;5,1 трлн руб. (+16% г/г)</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>03.06.2026</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>https://1prime.ru/20260603/vtb-870441128.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>ВТБ</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — прямая цитата официального лица, ПМЭФ-2026</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Объём выдач ипотеки</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>1-е полугодие 2026</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>~2,1 трлн руб. (+40% г/г)</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>03.06.2026</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>https://1prime.ru/20260603/vtb-870441128.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>ДОМ.РФ</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Первичный, но без точных цифр — офиц. пост аккаунта dom.rf</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Ключевая ставка / риск для рынка</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Риск-сценарий</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Если средняя ставка за год выше 13–15% — давление на застройщиков, замедление выдачи ипотеки</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>09.02.2026</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tbank.ru/invest/social/profile/DOM.RF/e6b380da-3434-46cf-94d6-83c6bc5c386d/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F23"/>
+  <autoFilter ref="A1:H26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Make source links clickable and remove blue header fill in forecast table
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Прогнозы банков по ипотеке.xlsx
+++ b/Прогнозы банков по ипотеке.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +30,13 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -58,12 +65,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -445,42 +458,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Банк / источник</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Тип источника</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Показатель</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Период прогноза</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Сценарий</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Прогнозное значение</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Дата публикации</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Ссылка на первоисточник</t>
         </is>
@@ -522,7 +535,7 @@
           <t>31.08.2026</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
         </is>
@@ -564,7 +577,7 @@
           <t>31.08.2026</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
         </is>
@@ -606,7 +619,7 @@
           <t>31.08.2026</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
         </is>
@@ -648,7 +661,7 @@
           <t>31.08.2026</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
         </is>
@@ -690,7 +703,7 @@
           <t>31.08.2026</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
         </is>
@@ -732,7 +745,7 @@
           <t>31.08.2026</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
         </is>
@@ -774,7 +787,7 @@
           <t>31.08.2026</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
         </is>
@@ -816,7 +829,7 @@
           <t>07.05.2026</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>https://www.cbr.ru/dkp/mp_dec/decision_key_rate/comment_07052026/</t>
         </is>
@@ -858,7 +871,7 @@
           <t>07.05.2026</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>https://www.cbr.ru/dkp/mp_dec/decision_key_rate/comment_07052026/</t>
         </is>
@@ -900,7 +913,7 @@
           <t>07.05.2026</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>https://www.cbr.ru/dkp/mp_dec/decision_key_rate/comment_07052026/</t>
         </is>
@@ -942,7 +955,7 @@
           <t>н/д (ОНЕДКП 2026-2028)</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>https://www.cbr.ru/about_br/publ/ondkp/on_2026_2028/</t>
         </is>
@@ -984,7 +997,7 @@
           <t>н/д (ОНЕДКП 2026-2028)</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>https://www.cbr.ru/about_br/publ/ondkp/on_2026_2028/</t>
         </is>
@@ -1026,7 +1039,7 @@
           <t>н/д (публикация действует на 2026 год)</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
         </is>
@@ -1068,7 +1081,7 @@
           <t>н/д</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
         </is>
@@ -1110,7 +1123,7 @@
           <t>н/д</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
         </is>
@@ -1152,7 +1165,7 @@
           <t>н/д</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
         </is>
@@ -1194,7 +1207,7 @@
           <t>н/д</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
         </is>
@@ -1236,7 +1249,7 @@
           <t>н/д</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>https://raexpert.ru/researches/banks/ipoteka_2026/</t>
         </is>
@@ -1278,7 +1291,7 @@
           <t>н/д</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>https://raexpert.ru/researches/banks/ipoteka_2026/</t>
         </is>
@@ -1320,7 +1333,7 @@
           <t>н/д</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>https://raexpert.ru/researches/banks/ipoteka_2026/</t>
         </is>
@@ -1362,7 +1375,7 @@
           <t>н/д</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>https://raexpert.ru/researches/banks/bank_forecast_2026/</t>
         </is>
@@ -1404,7 +1417,7 @@
           <t>н/д</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>https://raexpert.ru/researches/banks/bank_forecast_2026/</t>
         </is>
@@ -1446,7 +1459,7 @@
           <t>03.06.2026</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>https://1prime.ru/20260603/vtb-870441128.html</t>
         </is>
@@ -1488,7 +1501,7 @@
           <t>03.06.2026</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>https://1prime.ru/20260603/vtb-870441128.html</t>
         </is>
@@ -1530,7 +1543,7 @@
           <t>09.02.2026</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>https://www.tbank.ru/invest/social/profile/DOM.RF/e6b380da-3434-46cf-94d6-83c6bc5c386d/</t>
         </is>
@@ -1538,6 +1551,33 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:H26"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId25"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Expand forecast table with mortgage-specific rates/volumes and subsidized mortgage data
Добавил отдельные листы «Ипотечные ставки и объёмы» (НКР, Сбербанк/Домклик, ВТБ, Эксперт РА, Frank RG) и «Льготная ипотека» (Минфин, НКР) на основе первичных источников, отдельно от ключевой ставки ЦБ.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Прогнозы банков по ипотеке.xlsx
+++ b/Прогнозы банков по ипотеке.xlsx
@@ -7,10 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прогнозы (первоисточники)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ипотечные ставки и объёмы" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Льготная ипотека" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ключевая ставка ЦБ (справочно)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Прогнозы (первоисточники)'!$A$1:$H$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ипотечные ставки и объёмы'!$A$1:$H$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Льготная ипотека'!$A$1:$H$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ключевая ставка ЦБ (справочно)'!$A$1:$H$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,28 +33,18 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <color rgb="000563C1"/>
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -65,18 +59,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -444,56 +435,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Банк / источник</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Тип источника</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Показатель</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>Период прогноза</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Сценарий</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Прогнозное значение</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Период</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Сценарий / условие</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Дата публикации</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Ссылка на первоисточник</t>
         </is>
@@ -502,620 +493,620 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Банк России (ЦБ РФ)</t>
+          <t>НКР (рейтинговое агентство)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Первичный — офиц. документ</t>
+          <t>Первичный — аналитический отчёт</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка (среднегодовая)</t>
+          <t>Средневзвешенная ставка по новым ипотечным кредитам (с учётом господдержки)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2023 (факт)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Базовый</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>14,5–14,6%</t>
+          <t>7,9%</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>31.08.2026</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Банк России (ЦБ РФ)</t>
+          <t>НКР (рейтинговое агентство)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Первичный — офиц. документ</t>
+          <t>Первичный — аналитический отчёт</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка (среднегодовая)</t>
+          <t>Средневзвешенная ставка по новым ипотечным кредитам (с учётом господдержки)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>2024 (факт)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Базовый</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>10,5–12,5%</t>
+          <t>8,5%</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>31.08.2026</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Банк России (ЦБ РФ)</t>
+          <t>НКР (рейтинговое агентство)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Первичный — офиц. документ</t>
+          <t>Первичный — аналитический отчёт</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка (среднегодовая)</t>
+          <t>Средневзвешенная ставка по новым ипотечным кредитам (с учётом господдержки)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2028</t>
+          <t>2025 (факт)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Базовый</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>8,0–9,0%</t>
+          <t>7,6%</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>31.08.2026</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Банк России (ЦБ РФ)</t>
+          <t>НКР (рейтинговое агентство)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Первичный — офиц. документ</t>
+          <t>Первичный — аналитический отчёт</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка (среднегодовая)</t>
+          <t>Средневзвешенная ставка по новым ипотечным кредитам (с учётом господдержки)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2029</t>
+          <t>2026 (прогноз)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Базовый</t>
+          <t>Базовый сценарий НКР: ключевая ставка ЦБ 14–14,5% в среднем за год</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>7,5–8,5%</t>
+          <t>10,5–11,5% (рост объясняется падением доли льготных программ, а не удорожанием рынка)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>31.08.2026</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Банк России (ЦБ РФ)</t>
+          <t>НКР (рейтинговое агентство)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Первичный — офиц. документ</t>
+          <t>Первичный — аналитический отчёт (факт)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка (среднегодовая)</t>
+          <t>Средняя ставка новых выдач</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>Апрель 2026 (факт)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Дезинфляционный</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>9,0–11,0%</t>
+          <t>10,3% (максимум с 2019 года)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>31.08.2026</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Банк России (ЦБ РФ)</t>
+          <t>НКР (рейтинговое агентство)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Первичный — офиц. документ</t>
+          <t>Первичный — аналитический отчёт</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка (среднегодовая)</t>
+          <t>Объём выдачи ипотеки (весь рынок)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>2026 (прогноз)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Проинфляционный</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>13,0–15,0%</t>
+          <t>4,7–5,1 трлн руб. (+7–14% г/г)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>31.08.2026</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Банк России (ЦБ РФ)</t>
+          <t>НКР (рейтинговое агентство)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Первичный — офиц. документ</t>
+          <t>Первичный — аналитический отчёт</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка (среднегодовая)</t>
+          <t>Количество выданных кредитов</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>2026 (прогноз)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Рисковый</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>19,0–21,0%</t>
+          <t>1,0–1,1 млн (+7–10% г/г)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>31.08.2026</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Банк России (ЦБ РФ)</t>
+          <t>НКР (рейтинговое агентство)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Первичный — офиц. документ (более ранняя оценка)</t>
+          <t>Первичный — аналитический отчёт</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка (среднегодовая)</t>
+          <t>Ипотечный портфель (остаток)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2026 (прогноз)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Базовый</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>14,0–14,5%</t>
+          <t>22,5–23,3 трлн руб. (+8–12% г/г)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>07.05.2026</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.cbr.ru/dkp/mp_dec/decision_key_rate/comment_07052026/</t>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Банк России (ЦБ РФ)</t>
+          <t>НКР (рейтинговое агентство)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Первичный — офиц. документ (более ранняя оценка)</t>
+          <t>Первичный — аналитический отчёт</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка (среднегодовая)</t>
+          <t>Средний чек ипотечного кредита</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>2026 (прогноз)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Базовый</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>8,0–10,0%</t>
+          <t>4,4–4,6 млн руб.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>07.05.2026</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>https://www.cbr.ru/dkp/mp_dec/decision_key_rate/comment_07052026/</t>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Банк России (ЦБ РФ)</t>
+          <t>ДОМ.РФ (М. Гольдберг, рук. Аналитического центра)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Первичный — офиц. документ (более ранняя оценка)</t>
+          <t>Первичный — совместный отчёт НКР/ДОМ.РФ/ЕРЗ</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка (среднегодовая)</t>
+          <t>Порог рыночной ставки ипотеки, при котором рассрочка перестанет быть массовым инструментом</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2028</t>
+          <t>Ориентир без указания года</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Базовый</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>7,5–8,5%</t>
+          <t>~12% годовых</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>07.05.2026</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>https://www.cbr.ru/dkp/mp_dec/decision_key_rate/comment_07052026/</t>
+          <t>15.04.2026</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/corps/NCR_Dom.rf_ERZ_Real_Estate_Apr_26.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Банк России (ЦБ РФ)</t>
+          <t>ЕРЗ (К. Холопик, руководитель)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Первичный — офиц. документ (предыдущий цикл)</t>
+          <t>Первичный — совместный отчёт НКР/ДОМ.РФ/ЕРЗ</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка (среднегодовая)</t>
+          <t>Порог ключевой ставки ЦБ, при котором начнёт оживать рыночная ипотека</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>Ориентир без указания года</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Базовый</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>13,0–15,0%</t>
+          <t>&lt;10%</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>н/д (ОНЕДКП 2026-2028)</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2026_2028/</t>
+          <t>15.04.2026</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/corps/NCR_Dom.rf_ERZ_Real_Estate_Apr_26.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Банк России (ЦБ РФ)</t>
+          <t>Сбербанк</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Первичный — офиц. документ (предыдущий цикл)</t>
+          <t>Первичный — пресс-центр sberbank.ru</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка (среднегодовая)</t>
+          <t>Объём выдач ипотеки (весь рынок РФ)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>2026 (первоначальный прогноз)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Базовый</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>7,5–8,5%</t>
+          <t>5,6 трлн руб. (+40% г/г)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>н/д (ОНЕДКП 2026-2028)</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2026_2028/</t>
+          <t>13.07.2026</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sberbank.ru/ru/sberpress/all/article?newsID=021809fd-e899-4c43-a554-7a12c5c93e2c&amp;blockID=1303&amp;regionID=77&amp;lang=ru&amp;type=NEWS</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>SberCIB (аналитика Сбербанка)</t>
+          <t>Сбербанк</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Первичный — сайт SberCIB</t>
+          <t>Первичный — пресс-центр sberbank.ru (факт)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка</t>
+          <t>Объём выдач ипотеки (весь рынок)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Сентябрь 2026</t>
+          <t>1-е полугодие 2026 (факт)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Базовый</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>~1,6 трлн руб. (+71,5% г/г)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>н/д (публикация действует на 2026 год)</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
+          <t>13.07.2026</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sberbank.ru/ru/sberpress/all/article?newsID=021809fd-e899-4c43-a554-7a12c5c93e2c&amp;blockID=1303&amp;regionID=77&amp;lang=ru&amp;type=NEWS</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>SberCIB (аналитика Сбербанка)</t>
+          <t>Домклик (Сбербанк)</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Первичный — сайт SberCIB</t>
+          <t>Первичный — собственный блог blog.domclick.ru</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка</t>
+          <t>Объём выдач ипотеки (весь рынок, пересмотрено вниз)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Октябрь 2026</t>
+          <t>2026 (уточнённый прогноз)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Базовый</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>13,75%</t>
+          <t>5 трлн руб. (снижено с 5,6 трлн)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>н/д</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
+          <t>н/д (после 13.07.2026)</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>https://blog.domclick.ru/novosti/post/chto-zhdet-rynok-nedvizhimosti-i-ipoteki-v-2026-godu-prognozy-glavy-domklik</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>SberCIB (аналитика Сбербанка)</t>
+          <t>Домклик (Сбербанк)</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Первичный — сайт SberCIB</t>
+          <t>Первичный — собственный блог blog.domclick.ru</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка</t>
+          <t>Ежемесячный объём выдач рыночной ипотеки</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Ноябрь 2026</t>
+          <t>4-й квартал 2026</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Базовый</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>13,75%</t>
+          <t>~200 млрд руб./мес.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1123,110 +1114,110 @@
           <t>н/д</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>https://blog.domclick.ru/novosti/post/chto-zhdet-rynok-nedvizhimosti-i-ipoteki-v-2026-godu-prognozy-glavy-domklik</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>SberCIB (аналитика Сбербанка)</t>
+          <t>ВТБ</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Первичный — сайт SberCIB</t>
+          <t>Первичный — прямая цитата ст. вице-президента А. Охорзина, зафиксировано ТАСС</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка</t>
+          <t>Ставка по рыночной (без господдержки) ипотеке</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Декабрь 2026</t>
+          <t>Конец 2026</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Базовый</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>13,5%</t>
+          <t>16–17%</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>н/д</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
+          <t>н/д (2026)</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>https://tass.ru/ekonomika/27658353</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>SberCIB (аналитика Сбербанка)</t>
+          <t>ВТБ</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Первичный — сайт SberCIB</t>
+          <t>Первичный — прямая цитата А. Охорзина, зафиксировано ТАСС</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Ключевая ставка (среднегодовая)</t>
+          <t>Доля рыночной ипотеки в выдачах ВТБ</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>С июля 2026, ежемесячно</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Базовый</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>14,5%</t>
+          <t>&gt;50%</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>н/д</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
+          <t>н/д (2026)</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>https://tass.ru/ekonomika/27658353</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Эксперт РА</t>
+          <t>ВТБ</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Первичный — исследование агентства</t>
+          <t>Первичный — прямая цитата ст. вице-президента А. Охорзина, ПМЭФ-2026, зафиксировано ПРАЙМ</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Объём выдач ипотеки</t>
+          <t>Объём выдач ипотеки (весь рынок РФ)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1241,17 +1232,17 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Рост на 15–20% г/г, свыше 5 трлн руб.</t>
+          <t>&gt;5,1 трлн руб. (+16% г/г)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>н/д</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>https://raexpert.ru/researches/banks/ipoteka_2026/</t>
+          <t>03.06.2026</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>https://1prime.ru/20260603/vtb-870441128.html</t>
         </is>
       </c>
     </row>
@@ -1268,12 +1259,12 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Доля льготной ипотеки в выдачах</t>
+          <t>Ставка по ипотеке на первичном/вторичном рынке (факт, без субсидий)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>1-е полугодие 2026</t>
+          <t>Середина января 2026</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1283,7 +1274,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Выше 50%</t>
+          <t>21,25% / 21,22%</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1291,7 +1282,7 @@
           <t>н/д</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>https://raexpert.ru/researches/banks/ipoteka_2026/</t>
         </is>
@@ -1310,12 +1301,12 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Доля льготной ипотеки в выдачах</t>
+          <t>Ставка по рыночной ипотеке (без субсидий)</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>2-е полугодие 2026</t>
+          <t>1-е полугодие 2026</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1325,7 +1316,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Паритет с рыночной (~50%)</t>
+          <t>17–21%</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1333,7 +1324,7 @@
           <t>н/д</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>https://raexpert.ru/researches/banks/ipoteka_2026/</t>
         </is>
@@ -1347,27 +1338,27 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Первичный — исследование агентства (др. отчёт)</t>
+          <t>Первичный — исследование агентства</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Объём выдач ипотеки</t>
+          <t>Ставка по рыночной ипотеке (без субсидий)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>Конец 2026</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>При условии ускорения смягчения ДКП со 2-го полугодия</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>До 6,2 трлн руб. (1,2 млн кредитов), +59% г/г</t>
+          <t>До 15%</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1375,41 +1366,41 @@
           <t>н/д</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>https://raexpert.ru/researches/banks/bank_forecast_2026/</t>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>https://raexpert.ru/researches/banks/ipoteka_2026/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Эксперт РА</t>
+          <t>Frank RG</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Первичный — исследование агентства (др. отчёт, для сравнения)</t>
+          <t>Первичный — собственное исследование агентства</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Объём выдач ипотеки</t>
+          <t>Ставка по рыночной ипотеке (без субсидий)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2025 (факт/оценка)</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>При снижении ключевой ставки ЦБ до 13–14%</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>3,9 трлн руб., −20% г/г</t>
+          <t>14,5–15% (точка активизации спроса на первичке)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1417,140 +1408,14 @@
           <t>н/д</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>https://raexpert.ru/researches/banks/bank_forecast_2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>ВТБ</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Первичный — прямая цитата официального лица (ст. вице-президент А. Охорзин), ПМЭФ-2026; зафиксировано информагентством ПРАЙМ, т.к. отдельного пресс-релиза на vtb.ru не найдено</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Объём выдач ипотеки</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>&gt;5,1 трлн руб. (+16% г/г)</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>03.06.2026</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>https://1prime.ru/20260603/vtb-870441128.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>ВТБ</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Первичный — прямая цитата официального лица, ПМЭФ-2026</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Объём выдач ипотеки</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>1-е полугодие 2026</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>~2,1 трлн руб. (+40% г/г)</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>03.06.2026</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>https://1prime.ru/20260603/vtb-870441128.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>ДОМ.РФ</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Первичный, но без точных цифр — офиц. пост аккаунта dom.rf</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Ключевая ставка / риск для рынка</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Риск-сценарий</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Если средняя ставка за год выше 13–15% — давление на застройщиков, замедление выдачи ипотеки</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>09.02.2026</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>https://www.tbank.ru/invest/social/profile/DOM.RF/e6b380da-3434-46cf-94d6-83c6bc5c386d/</t>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>https://frankrg.com/news/ipoteka-2025-2026-stress-test-vysokimi-stavkami-i-prognozy-na-vosstanovlenie</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H26"/>
+  <autoFilter ref="A1:H23"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
@@ -1574,9 +1439,1305 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId25"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Банк / источник</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Тип источника</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Показатель</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Период</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Сценарий / условие</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Дата публикации</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Ссылка на первоисточник</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Минфин РФ</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — пресс-центр minfin.gov.ru</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Условия «Семейной ипотеки»: ставка / срок программы</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>До 2030 года</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Ставка 6% годовых для семей с ребёнком до 6 лет; первонач. взнос 20%</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>10.07.2024</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>https://minfin.gov.ru/ru/press-center?id_4=39161</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Минфин РФ</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — пресс-центр minfin.gov.ru</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Лимит суммы «Семейной ипотеки» (Москва/СПб и области)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>До 2030 года</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>В программе / с рыночной надбавкой</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>до 12 млн руб. / до 30 млн руб.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>10.07.2024</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>https://minfin.gov.ru/ru/press-center?id_4=39161</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Минфин РФ</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — пресс-центр minfin.gov.ru</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Лимит суммы «Семейной ипотеки» (остальные регионы)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>До 2030 года</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>В программе / с рыночной надбавкой</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>до 6 млн руб. / до 15 млн руб.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>10.07.2024</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>https://minfin.gov.ru/ru/press-center?id_4=39161</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Минфин РФ</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — пресс-центр minfin.gov.ru</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Бюджетные ассигнования на субсидирование «Семейной ипотеки»</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>По закону о федеральном бюджете 2025–2027</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>637,0 млрд руб.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>н/д</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>https://minfin.gov.ru/ru/press-center/?id_4=39540-o_limitakh_po_semeinoi_ipoteke</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Минфин РФ</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — пресс-центр minfin.gov.ru</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Бюджетные ассигнования на субсидирование «Семейной ипотеки»</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>По закону о федеральном бюджете 2025–2027</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>454,1 млрд руб.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>н/д</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>https://minfin.gov.ru/ru/press-center/?id_4=39540-o_limitakh_po_semeinoi_ipoteke</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Минфин РФ</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — пресс-центр minfin.gov.ru</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Бюджетные ассигнования на субсидирование «Семейной ипотеки»</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>По закону о федеральном бюджете 2025–2027</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>358,3 млрд руб.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>н/д</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>https://minfin.gov.ru/ru/press-center/?id_4=39540-o_limitakh_po_semeinoi_ipoteke</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Минфин РФ (А. Яковлев, директор департамента)</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — пресс-центр minfin.gov.ru</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Доля льготных программ в выдачах ипотеки (факт)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>По количеству / по сумме</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>63% / 80%</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>28.04.2026</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>https://minfin.gov.ru/ru/press-center/?id_4=40329-aleksei_yakovlev_po_mere_smyagcheniya_dkp_budet_vosstanavlivatsya_balans_mezhdu_rynochnoi_i_lgotnoi_ipotekoi</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Минфин РФ</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — пресс-центр minfin.gov.ru</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Тренд по балансу рыночной/льготной ипотеки</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026 и далее</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>По мере смягчения денежно-кредитной политики</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Постепенное восстановление баланса в пользу рыночных условий (без числовых прогнозов)</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>28.04.2026</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>https://minfin.gov.ru/ru/press-center/?id_4=40329-aleksei_yakovlev_po_mere_smyagcheniya_dkp_budet_vosstanavlivatsya_balans_mezhdu_rynochnoi_i_lgotnoi_ipotekoi</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>НКР (рейтинговое агентство)</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — аналитический отчёт</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Доля льготных программ в новых выдачах ипотеки</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2023 (факт)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>62%</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>НКР (рейтинговое агентство)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — аналитический отчёт</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Доля льготных программ в новых выдачах ипотеки</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2024 (факт)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>73%</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>НКР (рейтинговое агентство)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — аналитический отчёт</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Доля льготных программ в новых выдачах ипотеки</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2025 (факт)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>82%</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>НКР (рейтинговое агентство)</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — аналитический отчёт</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Доля льготных программ в новых выдачах ипотеки</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026 (прогноз, к концу года)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Впервые за 4 года</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>НКР (рейтинговое агентство)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — аналитический отчёт</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Доля льготных программ в новых выдачах ипотеки (факт, помесячно)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Февраль–март 2026 (факт)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>После ужесточения условий «Семейной ипотеки» с 1 февраля 2026</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Снижение с &gt;80% до 60%</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>НКР (рейтинговое агентство)</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — аналитический отчёт</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Ужесточение условий «Семейной ипотеки»</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Объявленные изменения параметров</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Повышение ставки до 10–12% для семей с 1–2 детьми; ограничение суммы кредита</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>НКР (рейтинговое агентство)</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — аналитический отчёт</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Доля рыночных (нельготных) программ в новых выдачах</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2027 (прогноз)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Не менее 50%, доля продолжит расти</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>НКР (рейтинговое агентство)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — аналитический отчёт</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Доля новых выдач с показателем долговой нагрузки (ПДН) свыше 80%</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>I квартал 2026 (факт)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>После ужесточения условий «Семейной ипотеки»</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Снижение до 4% (с 6% годом ранее и 33% двумя годами ранее)</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Эксперт РА</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — исследование агентства</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Доля льготной ипотеки в выдачах</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>1-е полугодие 2026</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Выше 50%</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>н/д</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>https://raexpert.ru/researches/banks/ipoteka_2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Эксперт РА</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — исследование агентства</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Доля льготной ипотеки в выдачах</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>2-е полугодие 2026</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Паритет с рыночной (~50%)</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>н/д</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>https://raexpert.ru/researches/banks/ipoteka_2026/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H19"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId18"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Банк / источник</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Тип источника</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Показатель</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Период</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Сценарий / условие</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Дата публикации</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Ссылка на первоисточник</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Банк России (ЦБ РФ)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — офиц. документ</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Ключевая ставка (среднегодовая)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Базовый</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>14,5–14,6%</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>31.08.2026</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Банк России (ЦБ РФ)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — офиц. документ</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Ключевая ставка (среднегодовая)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Базовый</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>10,5–12,5%</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>31.08.2026</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Банк России (ЦБ РФ)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — офиц. документ</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Ключевая ставка (среднегодовая)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Базовый</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>8,0–9,0%</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>31.08.2026</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Банк России (ЦБ РФ)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — офиц. документ</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Ключевая ставка (среднегодовая)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Базовый</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>7,5–8,5%</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>31.08.2026</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Банк России (ЦБ РФ)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — офиц. документ</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Ключевая ставка (среднегодовая)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Дезинфляционный</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>9,0–11,0%</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>31.08.2026</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Банк России (ЦБ РФ)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — офиц. документ</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Ключевая ставка (среднегодовая)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Проинфляционный</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>13,0–15,0%</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>31.08.2026</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Банк России (ЦБ РФ)</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — офиц. документ</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Ключевая ставка (среднегодовая)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Рисковый</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>19,0–21,0%</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>31.08.2026</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/about_br/publ/ondkp/on_2027_2029</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>НКР (рейтинговое агентство)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — собственное допущение для прогноза ипотеки</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Ключевая ставка (среднегодовая, допущение НКР)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Базовый сценарий НКР</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>14–14,5%</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>SberCIB (аналитика Сбербанка)</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — сайт SberCIB</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Ключевая ставка</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Сентябрь–декабрь 2026 (помесячно)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Базовый</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>14% → 13,75% → 13,75% → 13,5%</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>н/д</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>https://sbercib.ru/publication/prognoz-klyuchevoi-stavki-na-2026-god</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H10"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add NKR forecast for market-wide monthly mortgage issuance at end of 2026
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Прогнозы банков по ипотеке.xlsx
+++ b/Прогнозы банков по ипотеке.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2209,6 +2209,48 @@
       <c r="H42" s="3" t="inlineStr">
         <is>
           <t>https://наш.дом.рф/instructions/ipoteka-v-2026-2027-godakh-chto-proiskhodit-na-rynke/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>НКР (рейтинговое агентство)</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — аналитический отчёт</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Среднемесячный объём выдачи ипотеки (весь рынок)</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Конец 2026 (прогноз)</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Даже при ключевой ставке ЦБ 13%</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Может превысить 450 млрд руб./мес.</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>30.06.2026</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
         </is>
       </c>
     </row>
@@ -2256,6 +2298,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId42"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix наш.дом.рф links to use punycode form (Cyrillic IDN returned 403)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Прогнозы банков по ипотеке.xlsx
+++ b/Прогнозы банков по ипотеке.xlsx
@@ -2082,7 +2082,7 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>https://наш.дом.рф/instructions/ipoteka-v-2026-2027-godakh-chto-proiskhodit-na-rynke/</t>
+          <t>https://xn--h1alcedd.xn--d1aqf.xn--p1ai/instructions/ipoteka-v-2026-2027-godakh-chto-proiskhodit-na-rynke/</t>
         </is>
       </c>
     </row>
@@ -2124,7 +2124,7 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>https://наш.дом.рф/instructions/ipoteka-v-2026-2027-godakh-chto-proiskhodit-na-rynke/</t>
+          <t>https://xn--h1alcedd.xn--d1aqf.xn--p1ai/instructions/ipoteka-v-2026-2027-godakh-chto-proiskhodit-na-rynke/</t>
         </is>
       </c>
     </row>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>https://наш.дом.рф/instructions/ipoteka-v-2026-2027-godakh-chto-proiskhodit-na-rynke/</t>
+          <t>https://xn--h1alcedd.xn--d1aqf.xn--p1ai/instructions/ipoteka-v-2026-2027-godakh-chto-proiskhodit-na-rynke/</t>
         </is>
       </c>
     </row>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>https://наш.дом.рф/instructions/ipoteka-v-2026-2027-godakh-chto-proiskhodit-na-rynke/</t>
+          <t>https://xn--h1alcedd.xn--d1aqf.xn--p1ai/instructions/ipoteka-v-2026-2027-godakh-chto-proiskhodit-na-rynke/</t>
         </is>
       </c>
     </row>
@@ -3243,7 +3243,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>https://наш.дом.рф/instructions/ipoteka-v-2026-2027-godakh-chto-proiskhodit-na-rynke/</t>
+          <t>https://xn--h1alcedd.xn--d1aqf.xn--p1ai/instructions/ipoteka-v-2026-2027-godakh-chto-proiskhodit-na-rynke/</t>
         </is>
       </c>
     </row>
@@ -3285,7 +3285,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>https://наш.дом.рф/instructions/ipoteka-v-2026-2027-godakh-chto-proiskhodit-na-rynke/</t>
+          <t>https://xn--h1alcedd.xn--d1aqf.xn--p1ai/instructions/ipoteka-v-2026-2027-godakh-chto-proiskhodit-na-rynke/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix data-accuracy issues found in source cross-check
- Эксперт РА rate rows pointed at a raexpert.ru page that doesn't
  contain those figures; corrected to the actual source
  (raexpert.ru/researches/publications/rbc_jan19_2026/, 19.01.2026)
  and added the named analyst (Екатерина Щурихина).
- Сбербанк/Лейпи ИЖС monthly figures had April/May swapped relative
  to the Kommersant source wording.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Прогнозы банков по ипотеке.xlsx
+++ b/Прогнозы банков по ипотеке.xlsx
@@ -1249,12 +1249,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Эксперт РА</t>
+          <t>Эксперт РА (Е. Щурихина, директор по банковским рейтингам)</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Первичный — исследование агентства</t>
+          <t>Первичный — исследование, опубликовано на raexpert.ru (перепечатка материала РБК)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1279,24 +1279,24 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>19.01.2026</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>https://raexpert.ru/researches/banks/ipoteka_2026/</t>
+          <t>https://raexpert.ru/researches/publications/rbc_jan19_2026/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Эксперт РА</t>
+          <t>Эксперт РА (Е. Щурихина, директор по банковским рейтингам)</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Первичный — исследование агентства</t>
+          <t>Первичный — исследование, опубликовано на raexpert.ru (перепечатка материала РБК)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1321,24 +1321,24 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>19.01.2026</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>https://raexpert.ru/researches/banks/ipoteka_2026/</t>
+          <t>https://raexpert.ru/researches/publications/rbc_jan19_2026/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Эксперт РА</t>
+          <t>Эксперт РА (Е. Щурихина, директор по банковским рейтингам)</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Первичный — исследование агентства</t>
+          <t>Первичный — исследование, опубликовано на raexpert.ru (перепечатка материала РБК)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1363,12 +1363,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>19.01.2026</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>https://raexpert.ru/researches/banks/ipoteka_2026/</t>
+          <t>https://raexpert.ru/researches/publications/rbc_jan19_2026/</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Апрель–май 2026 (факт)</t>
+          <t>Май–апрель 2026 (факт)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>18 млрд и 17 млрд руб. в месяц (в 1,5–2 раза выше 2025 года)</t>
+          <t>18 млрд и 17 млрд руб. соответственно (в 1,5–2 раза выше 2025 года)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add 2027 mortgage forecast data (ДОМ.РФ corporate post)
Adds ДОМ.РФ's own 2027 forecast (1.6-1.8m loans / 6.5-7.3 trln rub,
market rate down to 10.5%) from its official T-Bank Pulse account,
clarified as market (non-subsidized) rate per user question.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Прогнозы банков по ипотеке.xlsx
+++ b/Прогнозы банков по ипотеке.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2251,6 +2251,90 @@
       <c r="H43" s="3" t="inlineStr">
         <is>
           <t>https://ratings.ru/files/research/banks/NCR_Mortgage_Jun2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>ДОМ.РФ (официальный корпоративный аккаунт на Т-Банк Инвестиции/Pulse)</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — корпоративный пост ДОМ.РФ</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Объём выдач ипотеки, весь рынок РФ (прогноз)</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>2027 (прогноз, опубликован 29.07.2025 — до цикла снижения ставок 2026 года, мог быть скорректирован более поздними материалами ДОМ.РФ)</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>1,6–1,8 млн кредитов на 6,5–7,3 трлн руб. (для сравнения 2026: 1,3–1,4 млн / 5,1–5,5 трлн)</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>29.07.2025</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tbank.ru/invest/social/profile/DOM.RF/7fb249e9-b726-449c-96ae-f308c8c4fc5e/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>ДОМ.РФ (официальный корпоративный аккаунт на Т-Банк Инвестиции/Pulse)</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Первичный — корпоративный пост ДОМ.РФ</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Ставка по рыночной ипотеке, без субсидий (прогноз)</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>2027 (прогноз, опубликован 29.07.2025 — см. примечание выше)</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>До 10,5%</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>29.07.2025</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tbank.ru/invest/social/profile/DOM.RF/7fb249e9-b726-449c-96ae-f308c8c4fc5e/</t>
         </is>
       </c>
     </row>
@@ -2299,6 +2383,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix mortgage-rate row misattributed to Frank RG
The 14.5-15% market-rate figure is a quote from Марина Заботина
(ПСБ), given at the Frank Mortgage Award 2025 ceremony and reported
by Frank RG, not Frank RG's own research.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Прогнозы банков по ипотеке.xlsx
+++ b/Прогнозы банков по ипотеке.xlsx
@@ -1375,12 +1375,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Frank RG</t>
+          <t>ПСБ — Марина Заботина, директор департамента ипотечного бизнеса ПСБ</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Первичный — собственное исследование агентства</t>
+          <t>Первичный — прямая цитата на церемонии Frank Mortgage Award 2025 (18.11.2025), зафиксировано Frank RG</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1405,7 +1405,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Fix wrong TASS link for VTB market-mortgage-share row
The "Доля рыночной ипотеки в выдачах ВТБ" row cited a TASS article
that only covers VTB's rate forecast, not market share. Replaced with
the actual primary source: VTB's 19.06.2026 press release quote,
recorded by RIA Novosti.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Прогнозы банков по ипотеке.xlsx
+++ b/Прогнозы банков по ипотеке.xlsx
@@ -1170,7 +1170,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Первичный — прямая цитата А. Охорзина, зафиксировано ТАСС</t>
+          <t>Первичный — прямая цитата ст. вице-президента А. Охорзина из пресс-релиза банка, зафиксировано РИА Новости</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1195,12 +1195,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>н/д (2026)</t>
+          <t>19.06.2026</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>https://tass.ru/ekonomika/27658353</t>
+          <t>https://crimea.ria.ru/20260619/vydachi-lgotnoy-i-rynochnoy-ipoteki-vtb-sravnyalis-1157001042.html</t>
         </is>
       </c>
     </row>

</xml_diff>